<commit_message>
save 25 02 2026
</commit_message>
<xml_diff>
--- a/4 четверть_9_JavaScript_Vue 3.xlsx
+++ b/4 четверть_9_JavaScript_Vue 3.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70B77FC4-025C-4E3C-AAAE-B023B33C954A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A1598B-45A4-45D4-A55C-982CA60106EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="192" yWindow="-216" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="База" sheetId="12" r:id="rId1"/>
     <sheet name="Vue Css" sheetId="13" r:id="rId2"/>
     <sheet name="Теория" sheetId="14" r:id="rId3"/>
-    <sheet name="template" sheetId="15" r:id="rId4"/>
+    <sheet name="Vue blank template" sheetId="15" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="288">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -5804,17 +5804,72 @@
     }
 });</t>
   </si>
+  <si>
+    <t xml:space="preserve">        changeText(scope, e, type=false) {
+            let dataName = (!type) ? 'usersDataFilteredComp' : 'ipAndPassArray';
+            let res = this[dataName].map(i =&gt; ({...i}));
+            let index = scope.$index;
+            let prop = scope.column.property;
+            res[index][prop] = e.target ? e.target.value : e;
+            this[dataName] = res;
+        },</t>
+  </si>
+  <si>
+    <t>Reflection</t>
+  </si>
+  <si>
+    <t>Удобно!</t>
+  </si>
+  <si>
+    <t>Поверхностное копирование - удобно!</t>
+  </si>
+  <si>
+    <r>
+      <t>let res = this[dataName].map(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>i =&gt; ({...i})</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>);</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -6117,10 +6172,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -6131,20 +6186,20 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -6153,75 +6208,75 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="23" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="49" fontId="7" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="49" fontId="8" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="10" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="10" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="11" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="11" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -6230,22 +6285,28 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6582,7 +6643,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V97"/>
+  <dimension ref="A2:V102"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -6752,873 +6813,895 @@
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="15"/>
+      <c r="B13" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A14" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-    </row>
-    <row r="14" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+    </row>
+    <row r="15" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B15" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C15" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+    <row r="16" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B16" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C16" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="16" spans="1:22" ht="72" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="13" t="s">
+    <row r="17" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A17" s="2"/>
+      <c r="B17" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="10" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="10" t="s">
         <v>65</v>
-      </c>
-      <c r="B17" s="12"/>
-      <c r="C17" s="9"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="30" t="s">
-        <v>201</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="9"/>
     </row>
-    <row r="19" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="30" t="s">
+        <v>201</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="9"/>
+    </row>
+    <row r="20" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="B20" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C20" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D20" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="31" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="31" t="s">
         <v>202</v>
       </c>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-    </row>
-    <row r="21" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A21" s="2"/>
       <c r="B21" s="15"/>
-      <c r="C21" s="29" t="s">
+      <c r="C21" s="15"/>
+    </row>
+    <row r="22" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A22" s="2"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="29" t="s">
         <v>203</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B22" s="12"/>
-      <c r="C22" s="9"/>
-    </row>
-    <row r="23" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="2" t="s">
+      <c r="B23" s="12"/>
+      <c r="C23" s="9"/>
+    </row>
+    <row r="24" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B24" s="12"/>
       <c r="C24" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="B25" s="12"/>
+      <c r="C25" s="13" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="14" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B26" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="C25" s="13"/>
-    </row>
-    <row r="26" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
+      <c r="C26" s="13"/>
+    </row>
+    <row r="27" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B26" s="13" t="s">
+      <c r="B27" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C27" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="B27" s="13"/>
-      <c r="C27" s="13" t="s">
+    <row r="28" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="B28" s="13"/>
+      <c r="C28" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D28" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="216" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
+    <row r="29" spans="1:4" ht="216" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B28" s="13" t="s">
+      <c r="B29" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C29" s="15" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="10" t="s">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B29" s="12"/>
-      <c r="C29" s="9"/>
-    </row>
-    <row r="30" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="12"/>
+      <c r="C30" s="9"/>
+    </row>
+    <row r="31" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B31" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C31" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="B31" s="12"/>
-      <c r="C31" s="13" t="s">
+    <row r="32" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="B32" s="12"/>
+      <c r="C32" s="13" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
+    <row r="33" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B33" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C33" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
+    <row r="34" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B33" s="13"/>
-      <c r="C33" s="13" t="s">
+      <c r="B34" s="13"/>
+      <c r="C34" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="B34" s="12"/>
-      <c r="C34" s="13" t="s">
+    <row r="35" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="B35" s="12"/>
+      <c r="C35" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="D35" s="2" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="10" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B35" s="12"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="2"/>
-    </row>
-    <row r="36" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
+      <c r="B36" s="12"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B37" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C37" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="D37" s="2" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="B37" s="12"/>
-      <c r="C37" s="15" t="s">
+    <row r="38" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="B38" s="12"/>
+      <c r="C38" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
+    <row r="39" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B38" s="13" t="s">
+      <c r="B39" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C39" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="D38" s="2"/>
-    </row>
-    <row r="39" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B39" s="12"/>
-      <c r="C39" s="2" t="s">
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="B40" s="12"/>
+      <c r="C40" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
+    <row r="41" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B40" s="13" t="s">
+      <c r="B41" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="C40" s="13" t="s">
+      <c r="C41" s="13" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="17" t="s">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="1" t="s">
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="B42" s="15" t="s">
+    <row r="43" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="B43" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="C42" s="15" t="s">
+      <c r="C43" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="D42" s="15" t="s">
+      <c r="D43" s="15" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="10" t="s">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B43" s="13"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="1" t="s">
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="1" t="s">
         <v>125</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="216" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B44" s="32" t="s">
-        <v>254</v>
-      </c>
-      <c r="C44" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="D44" s="42" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="216" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B45" s="32" t="s">
+        <v>254</v>
+      </c>
+      <c r="C45" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="D45" s="42" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="216" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B45" s="15" t="s">
+      <c r="B46" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="C45" s="15" t="s">
+      <c r="C46" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="D45" s="42" t="s">
+      <c r="D46" s="42" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" s="10" t="s">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="D47" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A47" s="26" t="s">
+    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="B48" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="C47" s="1" t="s">
+      <c r="C48" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="D47" s="1" t="s">
+      <c r="D48" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="4" t="s">
+    <row r="49" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B48" s="15" t="s">
+      <c r="B49" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="C48" s="15" t="s">
+      <c r="C49" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="D48" s="1" t="s">
+      <c r="D49" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A49" s="4" t="s">
+    <row r="50" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A50" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B49" s="2" t="s">
+      <c r="B50" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C49" s="15" t="s">
+      <c r="C50" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="D49" s="1" t="s">
+      <c r="D50" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="9" t="s">
+    <row r="51" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B50" s="15" t="s">
+      <c r="B51" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="C50" s="15" t="s">
+      <c r="C51" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="D50" s="1" t="s">
+      <c r="D51" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A51" s="4" t="s">
+    <row r="52" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A52" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B52" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="C51" s="15" t="s">
+      <c r="C52" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="D51" s="1" t="s">
+      <c r="D52" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A52" s="9" t="s">
+    <row r="53" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A53" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="B53" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C52" s="15" t="s">
+      <c r="C53" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="D52" s="2" t="s">
+      <c r="D53" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="15" t="s">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B54" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="C53" s="15" t="s">
+      <c r="C54" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="D53" s="15"/>
-    </row>
-    <row r="54" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A54" s="15" t="s">
+      <c r="D54" s="15"/>
+    </row>
+    <row r="55" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A55" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B55" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="C54" s="15" t="s">
+      <c r="C55" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="D54" s="15" t="s">
+      <c r="D55" s="15" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A55" s="15" t="s">
+    <row r="56" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A56" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B56" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="C55" s="15" t="s">
+      <c r="C56" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="D55" s="15" t="s">
+      <c r="D56" s="15" t="s">
         <v>179</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A56" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B56" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="C56" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A57" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B57" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="C57" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A58" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B57" s="15" t="s">
+      <c r="B58" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="C57" s="15" t="s">
+      <c r="C58" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="D57" s="1" t="s">
+      <c r="D58" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A58" s="9" t="s">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B59" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="C58" s="15" t="s">
+      <c r="C59" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="D58" s="1" t="s">
+      <c r="D59" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A59" s="9" t="s">
+    <row r="60" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A60" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B59" s="15" t="s">
+      <c r="B60" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="C59" s="15" t="s">
+      <c r="C60" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="D59" s="15"/>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A60" s="10" t="s">
+      <c r="D60" s="15"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A61" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="B60" s="15"/>
-      <c r="C60" s="15"/>
-      <c r="D60" s="15"/>
-    </row>
-    <row r="61" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="C61" s="15" t="s">
+      <c r="B61" s="15"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+    </row>
+    <row r="62" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C62" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="D61" s="15"/>
-    </row>
-    <row r="62" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A62" s="1" t="s">
+      <c r="D62" s="15"/>
+    </row>
+    <row r="63" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B63" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C62" s="29" t="s">
+      <c r="C63" s="29" t="s">
         <v>195</v>
       </c>
-      <c r="D62" s="15"/>
-    </row>
-    <row r="63" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A63" s="1" t="s">
+      <c r="D63" s="15"/>
+    </row>
+    <row r="64" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B63" s="2" t="s">
+      <c r="B64" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C63" s="15" t="s">
+      <c r="C64" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="D63" s="15"/>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A64" s="10" t="s">
+      <c r="D64" s="15"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A65" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="B64" s="15"/>
-      <c r="C64" s="15"/>
-      <c r="D64" s="15" t="s">
+      <c r="B65" s="15"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="15" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="30" t="s">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A66" s="30" t="s">
         <v>201</v>
       </c>
-      <c r="B65" s="12"/>
-      <c r="C65" s="9"/>
-    </row>
-    <row r="66" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A66" s="2" t="s">
+      <c r="B66" s="12"/>
+      <c r="C66" s="9"/>
+    </row>
+    <row r="67" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A67" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B66" s="15" t="s">
+      <c r="B67" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="C66" s="15" t="s">
+      <c r="C67" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="D66" s="1" t="s">
+      <c r="D67" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="31" t="s">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A68" s="31" t="s">
         <v>202</v>
       </c>
-      <c r="B67" s="15"/>
-      <c r="C67" s="15"/>
-    </row>
-    <row r="68" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A68" s="2"/>
       <c r="B68" s="15"/>
-      <c r="C68" s="29" t="s">
+      <c r="C68" s="15"/>
+    </row>
+    <row r="69" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A69" s="2"/>
+      <c r="B69" s="15"/>
+      <c r="C69" s="29" t="s">
         <v>203</v>
       </c>
-      <c r="D68" s="2" t="s">
+      <c r="D69" s="2" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A69" s="10" t="s">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A70" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="B69" s="15"/>
-      <c r="C69" s="15"/>
-      <c r="D69" s="1" t="s">
+      <c r="B70" s="15"/>
+      <c r="C70" s="15"/>
+      <c r="D70" s="1" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A70" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="C70" s="29" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C71" s="29" t="s">
-        <v>221</v>
-      </c>
-      <c r="D71" s="2"/>
+        <v>214</v>
+      </c>
     </row>
     <row r="72" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C72" s="29" t="s">
+        <v>221</v>
+      </c>
+      <c r="D72" s="2"/>
+    </row>
+    <row r="73" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="B72" s="29" t="s">
+      <c r="B73" s="29" t="s">
         <v>224</v>
       </c>
-      <c r="C72" s="29" t="s">
+      <c r="C73" s="29" t="s">
         <v>222</v>
       </c>
-      <c r="D72" s="2" t="s">
+      <c r="D73" s="2" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="73" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A73" s="2" t="s">
+    <row r="74" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B74" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="C73" s="29" t="s">
+      <c r="C74" s="29" t="s">
         <v>227</v>
       </c>
-      <c r="D73" s="2" t="s">
+      <c r="D74" s="2" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="74" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A74" s="2" t="s">
+    <row r="75" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A75" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B75" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="C74" s="29" t="s">
+      <c r="C75" s="29" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A75" s="2" t="s">
+    <row r="76" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B76" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="C75" s="29" t="s">
+      <c r="C76" s="29" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A76" s="1" t="s">
+    <row r="77" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A77" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B77" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="C76" s="32" t="s">
+      <c r="C77" s="32" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A77" s="1" t="s">
+    <row r="78" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A78" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B78" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="C77" s="29" t="s">
+      <c r="C78" s="29" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" s="10" t="s">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="D78" s="1" t="s">
+      <c r="D79" s="1" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A79" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="C79" s="9"/>
-      <c r="D79" s="2"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C80" s="9"/>
+      <c r="D80" s="2"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>252</v>
+        <v>235</v>
       </c>
       <c r="C81" s="9"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>236</v>
+        <v>253</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>252</v>
       </c>
       <c r="C82" s="9"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C83" s="9"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C84" s="9"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C85" s="9"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>240</v>
-      </c>
+        <v>239</v>
+      </c>
+      <c r="C86" s="9"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A88" s="2" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A88" s="32" t="s">
+    <row r="89" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A89" s="32" t="s">
         <v>247</v>
       </c>
-      <c r="B88" s="32"/>
-      <c r="C88" s="32" t="s">
+      <c r="B89" s="32"/>
+      <c r="C89" s="32" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A89" s="32" t="s">
+    <row r="90" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A90" s="32" t="s">
         <v>249</v>
       </c>
-      <c r="B89" s="32" t="s">
+      <c r="B90" s="32" t="s">
         <v>256</v>
       </c>
-      <c r="C89" s="32" t="s">
+      <c r="C90" s="32" t="s">
         <v>250</v>
       </c>
-      <c r="D89" s="32" t="s">
+      <c r="D90" s="32" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A90" s="1" t="s">
+    <row r="91" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A91" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="B90" s="32" t="s">
+      <c r="B91" s="32" t="s">
         <v>261</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="1" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="93" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A93" s="1" t="s">
+    <row r="94" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A94" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B93" s="32" t="s">
+      <c r="B94" s="32" t="s">
         <v>242</v>
       </c>
-      <c r="C93" s="32" t="s">
+      <c r="C94" s="32" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" s="1" t="s">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="B94" s="2" t="s">
+      <c r="B95" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="C94" s="33" t="s">
+      <c r="C95" s="33" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" s="34" t="s">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A96" s="34" t="s">
         <v>258</v>
       </c>
-      <c r="D95" s="1" t="s">
+      <c r="D96" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A96" s="1" t="s">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B96" s="2" t="s">
+      <c r="B97" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="C96" s="32" t="s">
+      <c r="C97" s="32" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A97" s="1" t="s">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B97" s="2" t="s">
+      <c r="B98" s="2" t="s">
         <v>263</v>
       </c>
     </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A101" s="10" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" ht="144" x14ac:dyDescent="0.3">
+      <c r="A102" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C102" s="44" t="s">
+        <v>283</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="15" type="noConversion"/>
+  <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -7663,10 +7746,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A1" s="43"/>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
+      <c r="A1" s="45"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="22"/>
@@ -8030,7 +8113,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C30:D44">
     <sortCondition ref="D30:D44"/>
   </sortState>
-  <phoneticPr fontId="15" type="noConversion"/>
+  <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -8096,7 +8179,7 @@
     <row r="4" spans="1:22" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A4" s="38"/>
       <c r="B4" s="38"/>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="43" t="s">
         <v>282</v>
       </c>
     </row>

</xml_diff>

<commit_message>
save 02 03 2026
</commit_message>
<xml_diff>
--- a/4 четверть_9_JavaScript_Vue 3.xlsx
+++ b/4 четверть_9_JavaScript_Vue 3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A1598B-45A4-45D4-A55C-982CA60106EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AA9107-EF8D-4D1D-B314-FA3DFC0BF592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="192" yWindow="-216" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="База" sheetId="12" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="290">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -2582,66 +2582,6 @@
   </si>
   <si>
     <t xml:space="preserve">Вариант 3 - стрелочная функция без return </t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Пояснение - удобно!</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Если мы опускаем return , значит внутри фигурных скобок уже </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>не стэк вызова функции</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>а сам object, который мы возвращаем в return</t>
-    </r>
   </si>
   <si>
     <t>data() { return {}}</t>
@@ -5851,17 +5791,179 @@
       <t>);</t>
     </r>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Пояснение - удобно!</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Если мы опускаем return , значит внутри фигурных скобок уже </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>не стэк вызова функции</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">а сам object, который мы возвращаем в return
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Важно - неудобно!</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Если в data есть обращение через this, то будет ошибка или не будет работать вообще! Так как this в стрелочной функции определяется в момент обращения к ней</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Не будет работать</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    data: () =&gt; ({
+        colorTypes: [{
+            value: 'notmo',
+            label</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: this.$t('noMoreThanDays')</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+        }, {
+...
+        },
+    }),</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="29" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -6172,10 +6274,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -6186,20 +6288,20 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -6208,75 +6310,75 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="24" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="49" fontId="8" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="49" fontId="9" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="10" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="10" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="11" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="11" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -6285,25 +6387,28 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -6643,7 +6748,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V102"/>
+  <dimension ref="A2:V103"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -6767,7 +6872,7 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -6783,7 +6888,7 @@
         <v>55</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
@@ -6795,913 +6900,922 @@
         <v>156</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="B12" s="15" t="s">
-        <v>159</v>
+      <c r="B12" s="47" t="s">
+        <v>287</v>
       </c>
       <c r="C12" s="15" t="s">
         <v>155</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A13" s="15"/>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="47" t="s">
+        <v>288</v>
+      </c>
+      <c r="C13" s="47" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A14" s="15"/>
+      <c r="B14" s="33" t="s">
+        <v>285</v>
+      </c>
+      <c r="C14" s="45" t="s">
         <v>286</v>
       </c>
-      <c r="C13" s="46" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A14" s="10" t="s">
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-    </row>
-    <row r="15" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+    </row>
+    <row r="16" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B16" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C16" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+    <row r="17" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B17" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C17" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
-      <c r="B17" s="13" t="s">
+    <row r="18" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A18" s="2"/>
+      <c r="B18" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="10" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="10" t="s">
         <v>65</v>
-      </c>
-      <c r="B18" s="12"/>
-      <c r="C18" s="9"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="30" t="s">
-        <v>201</v>
       </c>
       <c r="B19" s="12"/>
       <c r="C19" s="9"/>
     </row>
-    <row r="20" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="B20" s="12"/>
+      <c r="C20" s="9"/>
+    </row>
+    <row r="21" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B21" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="C21" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="C20" s="15" t="s">
-        <v>192</v>
-      </c>
-      <c r="D20" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="31" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="31" t="s">
+        <v>201</v>
+      </c>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+    </row>
+    <row r="23" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A23" s="2"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="29" t="s">
         <v>202</v>
       </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-    </row>
-    <row r="22" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A22" s="2"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="29" t="s">
+      <c r="D23" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="10" t="s">
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="9"/>
-    </row>
-    <row r="24" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
+      <c r="B24" s="12"/>
+      <c r="C24" s="9"/>
+    </row>
+    <row r="25" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B24" s="12"/>
-      <c r="C24" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B25" s="12"/>
       <c r="C25" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="B26" s="12"/>
+      <c r="C26" s="13" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="14" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="16" t="s">
+      <c r="B27" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="C26" s="13"/>
-    </row>
-    <row r="27" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
+      <c r="C27" s="13"/>
+    </row>
+    <row r="28" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B27" s="13" t="s">
+      <c r="B28" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C28" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D28" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="B28" s="13"/>
-      <c r="C28" s="13" t="s">
+    <row r="29" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="B29" s="13"/>
+      <c r="C29" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D29" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="216" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
+    <row r="30" spans="1:4" ht="216" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B30" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C30" s="15" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="10" t="s">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="12"/>
-      <c r="C30" s="9"/>
-    </row>
-    <row r="31" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="12"/>
+      <c r="C31" s="9"/>
+    </row>
+    <row r="32" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B32" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C32" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D32" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="B32" s="12"/>
-      <c r="C32" s="13" t="s">
+    <row r="33" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="B33" s="12"/>
+      <c r="C33" s="13" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
+    <row r="34" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="B34" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C34" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+    <row r="35" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B34" s="13"/>
-      <c r="C34" s="13" t="s">
+      <c r="B35" s="13"/>
+      <c r="C35" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="B35" s="12"/>
-      <c r="C35" s="13" t="s">
+    <row r="36" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="B36" s="12"/>
+      <c r="C36" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="10" t="s">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="B36" s="12"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="2"/>
-    </row>
-    <row r="37" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
+      <c r="B37" s="12"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B37" s="13" t="s">
+      <c r="B38" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="C37" s="13" t="s">
+      <c r="C38" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D38" s="2" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="B38" s="12"/>
-      <c r="C38" s="15" t="s">
+    <row r="39" spans="1:4" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="B39" s="12"/>
+      <c r="C39" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="D39" s="2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
+    <row r="40" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B39" s="13" t="s">
+      <c r="B40" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="C39" s="13" t="s">
+      <c r="C40" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="D39" s="2"/>
-    </row>
-    <row r="40" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B40" s="12"/>
-      <c r="C40" s="2" t="s">
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="B41" s="12"/>
+      <c r="C41" s="2" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
+    <row r="42" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B41" s="13" t="s">
+      <c r="B42" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="13" t="s">
+      <c r="C42" s="13" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="17" t="s">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="B42" s="13"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="1" t="s">
+      <c r="B43" s="13"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="B43" s="15" t="s">
+    <row r="44" spans="1:4" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="B44" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="C43" s="15" t="s">
+      <c r="C44" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="D43" s="15" t="s">
+      <c r="D44" s="15" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="10" t="s">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B44" s="13"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="1" t="s">
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="1" t="s">
         <v>125</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="216" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B45" s="32" t="s">
-        <v>254</v>
-      </c>
-      <c r="C45" s="15" t="s">
-        <v>77</v>
-      </c>
-      <c r="D45" s="42" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="216" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B46" s="32" t="s">
+        <v>253</v>
+      </c>
+      <c r="C46" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="D46" s="42" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="216" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B46" s="15" t="s">
+      <c r="B47" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="C46" s="15" t="s">
+      <c r="C47" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="D46" s="42" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="10" t="s">
+      <c r="D47" s="42" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D47" s="1" t="s">
+      <c r="D48" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A48" s="26" t="s">
+    <row r="49" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="15" t="s">
+      <c r="B49" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A50" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B50" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="C50" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="C48" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A49" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B49" s="15" t="s">
+      <c r="D50" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A52" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B52" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="C49" s="15" t="s">
-        <v>166</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A50" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="C50" s="15" t="s">
-        <v>167</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A51" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B51" s="15" t="s">
+      <c r="C52" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="C51" s="15" t="s">
+      <c r="D52" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A53" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="D51" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A52" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B52" s="2" t="s">
+      <c r="C53" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="C52" s="15" t="s">
+      <c r="D53" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A54" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="C54" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="D52" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A53" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="C53" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="D53" s="2" t="s">
+      <c r="D54" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="15" t="s">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="15" t="s">
         <v>131</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="C54" s="15" t="s">
-        <v>199</v>
-      </c>
-      <c r="D54" s="15"/>
-    </row>
-    <row r="55" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A55" s="15" t="s">
-        <v>90</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>177</v>
       </c>
       <c r="C55" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="D55" s="15"/>
+    </row>
+    <row r="56" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A56" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D55" s="15" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A56" s="15" t="s">
+      <c r="C56" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="D56" s="15" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A57" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="C56" s="15" t="s">
+      <c r="B57" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="D56" s="15" t="s">
+      <c r="C57" s="15" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A57" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B57" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="C57" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>25</v>
+      <c r="D57" s="15" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A58" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B58" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A59" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B58" s="15" t="s">
+      <c r="B59" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="C59" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C60" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A61" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B61" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="C61" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="D61" s="15"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A62" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="B62" s="15"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="15"/>
+    </row>
+    <row r="63" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C63" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="D63" s="15"/>
+    </row>
+    <row r="64" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C64" s="29" t="s">
+        <v>194</v>
+      </c>
+      <c r="D64" s="15"/>
+    </row>
+    <row r="65" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="C65" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="D65" s="15"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A66" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="B66" s="15"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="15" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="B67" s="12"/>
+      <c r="C67" s="9"/>
+    </row>
+    <row r="68" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B68" s="15" t="s">
         <v>190</v>
       </c>
-      <c r="C58" s="15" t="s">
-        <v>189</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="C59" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A60" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B60" s="15" t="s">
-        <v>188</v>
-      </c>
-      <c r="C60" s="15" t="s">
-        <v>187</v>
-      </c>
-      <c r="D60" s="15"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A61" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="B61" s="15"/>
-      <c r="C61" s="15"/>
-      <c r="D61" s="15"/>
-    </row>
-    <row r="62" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="C62" s="15" t="s">
-        <v>194</v>
-      </c>
-      <c r="D62" s="15"/>
-    </row>
-    <row r="63" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A63" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C63" s="29" t="s">
-        <v>195</v>
-      </c>
-      <c r="D63" s="15"/>
-    </row>
-    <row r="64" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A64" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="C64" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="D64" s="15"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="10" t="s">
+      <c r="C68" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" s="31" t="s">
+        <v>201</v>
+      </c>
+      <c r="B69" s="15"/>
+      <c r="C69" s="15"/>
+    </row>
+    <row r="70" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A70" s="2"/>
+      <c r="B70" s="15"/>
+      <c r="C70" s="29" t="s">
+        <v>202</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A71" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="B65" s="15"/>
-      <c r="C65" s="15"/>
-      <c r="D65" s="15" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="30" t="s">
-        <v>201</v>
-      </c>
-      <c r="B66" s="12"/>
-      <c r="C66" s="9"/>
-    </row>
-    <row r="67" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A67" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B67" s="15" t="s">
-        <v>191</v>
-      </c>
-      <c r="C67" s="15" t="s">
-        <v>192</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A68" s="31" t="s">
-        <v>202</v>
-      </c>
-      <c r="B68" s="15"/>
-      <c r="C68" s="15"/>
-    </row>
-    <row r="69" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="A69" s="2"/>
-      <c r="B69" s="15"/>
-      <c r="C69" s="29" t="s">
-        <v>203</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="B70" s="15"/>
-      <c r="C70" s="15"/>
-      <c r="D70" s="1" t="s">
+      <c r="B71" s="15"/>
+      <c r="C71" s="15"/>
+      <c r="D71" s="1" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A71" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="C71" s="29" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="72" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C72" s="29" t="s">
-        <v>221</v>
-      </c>
-      <c r="D72" s="2"/>
+        <v>213</v>
+      </c>
     </row>
     <row r="73" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C73" s="29" t="s">
+        <v>220</v>
+      </c>
+      <c r="D73" s="2"/>
+    </row>
+    <row r="74" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A74" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B74" s="29" t="s">
+        <v>223</v>
+      </c>
+      <c r="C74" s="29" t="s">
+        <v>221</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A75" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="B73" s="29" t="s">
+      <c r="B75" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="C73" s="29" t="s">
-        <v>222</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A74" s="2" t="s">
+      <c r="C75" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B74" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="C74" s="29" t="s">
+      <c r="B76" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C76" s="29" t="s">
         <v>227</v>
       </c>
-      <c r="D74" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A75" s="2" t="s">
+    </row>
+    <row r="77" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A77" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B77" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C77" s="29" t="s">
         <v>229</v>
       </c>
-      <c r="C75" s="29" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A76" s="2" t="s">
+    </row>
+    <row r="78" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A78" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C78" s="32" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A79" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="B79" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="C79" s="29" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A80" s="10" t="s">
         <v>231</v>
       </c>
-      <c r="C76" s="29" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A77" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="C77" s="32" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A78" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="C78" s="29" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A79" s="10" t="s">
+      <c r="D80" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="D79" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A80" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="C80" s="9"/>
-      <c r="D80" s="2"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C81" s="9"/>
+      <c r="D81" s="2"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>252</v>
+        <v>234</v>
       </c>
       <c r="C82" s="9"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
-        <v>236</v>
+        <v>252</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>251</v>
       </c>
       <c r="C83" s="9"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C84" s="9"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C85" s="9"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C86" s="9"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>240</v>
-      </c>
+        <v>238</v>
+      </c>
+      <c r="C87" s="9"/>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A89" s="32" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A89" s="2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A90" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="B90" s="32"/>
+      <c r="C90" s="32" t="s">
         <v>247</v>
       </c>
-      <c r="B89" s="32"/>
-      <c r="C89" s="32" t="s">
+    </row>
+    <row r="91" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A91" s="32" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A90" s="32" t="s">
+      <c r="B91" s="32" t="s">
+        <v>255</v>
+      </c>
+      <c r="C91" s="32" t="s">
         <v>249</v>
       </c>
-      <c r="B90" s="32" t="s">
+      <c r="D91" s="32" t="s">
         <v>256</v>
       </c>
-      <c r="C90" s="32" t="s">
-        <v>250</v>
-      </c>
-      <c r="D90" s="32" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A91" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="B91" s="32" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="92" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
-        <v>241</v>
+        <v>239</v>
+      </c>
+      <c r="B92" s="32" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="B95" s="32" t="s">
+        <v>241</v>
+      </c>
+      <c r="C95" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="B94" s="32" t="s">
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A96" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B96" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="C94" s="32" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="B95" s="2" t="s">
+      <c r="C96" s="33" t="s">
         <v>243</v>
       </c>
-      <c r="C95" s="33" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A96" s="34" t="s">
-        <v>258</v>
-      </c>
-      <c r="D96" s="1" t="s">
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A97" s="34" t="s">
+        <v>257</v>
+      </c>
+      <c r="D97" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A97" s="1" t="s">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A98" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B97" s="2" t="s">
+      <c r="B98" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C98" s="32" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A99" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B99" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="C97" s="32" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A98" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B98" s="2" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A101" s="10" t="s">
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A102" s="10" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" ht="144" x14ac:dyDescent="0.3">
+      <c r="A103" s="1" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" ht="144" x14ac:dyDescent="0.3">
-      <c r="A102" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="C102" s="44" t="s">
-        <v>283</v>
+      <c r="C103" s="44" t="s">
+        <v>282</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="16" type="noConversion"/>
+  <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -7746,10 +7860,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A1" s="45"/>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
+      <c r="A1" s="46"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="22"/>
@@ -7979,13 +8093,13 @@
     </row>
     <row r="6" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B6" s="32" t="s">
+        <v>264</v>
+      </c>
+      <c r="C6" s="32" t="s">
         <v>265</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="D6" s="1" t="s">
         <v>266</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
@@ -7995,13 +8109,13 @@
     </row>
     <row r="8" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B8" s="32" t="s">
+        <v>268</v>
+      </c>
+      <c r="C8" s="32" t="s">
+        <v>267</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>269</v>
-      </c>
-      <c r="C8" s="32" t="s">
-        <v>268</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
@@ -8011,38 +8125,38 @@
     </row>
     <row r="10" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C10" s="36" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:22" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="C11" s="36" t="s">
         <v>273</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="C11" s="36" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="144" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="288" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C13" s="36" t="s">
         <v>278</v>
-      </c>
-      <c r="C13" s="36" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
@@ -8113,7 +8227,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C30:D44">
     <sortCondition ref="D30:D44"/>
   </sortState>
-  <phoneticPr fontId="16" type="noConversion"/>
+  <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -8168,7 +8282,7 @@
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B3" s="38"/>
       <c r="C3" s="37"/>
@@ -8180,7 +8294,7 @@
       <c r="A4" s="38"/>
       <c r="B4" s="38"/>
       <c r="C4" s="43" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
save 19 03 2026
</commit_message>
<xml_diff>
--- a/4 четверть_9_JavaScript_Vue 3.xlsx
+++ b/4 четверть_9_JavaScript_Vue 3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AA9107-EF8D-4D1D-B314-FA3DFC0BF592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21E1E3B9-A8AA-48B2-B309-20F18B508861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="База" sheetId="12" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="291">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -2185,76 +2185,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">&lt;button 
-         v-bind:class="
-        {
-          </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>'btn-danger': colorEdit &amp;&amp; baseSettings.editUserCurrentSetting,
-          'btn-default': !colorEdit || !baseSettings.editUserCurrentSetting, 
-          'btn-primary': colorEdit &amp;&amp; !baseSettings.editUserCurrentSetting</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-         }
-       "
-&lt;/button&gt;</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">&lt;button 
-        v-bind:class="[
-           </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">'custom_class_1',
-            {'btn-danger': !colorEdit || !baseSettings.editUserCurrentSetting}, 
-           colorEdit &amp;&amp; baseSettings.editUserCurrentSetting ? 'btn-danger' : null </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-         ]"
-&lt;/button&gt;</t>
-    </r>
-  </si>
-  <si>
     <t>inline стили</t>
   </si>
   <si>
@@ -2331,34 +2261,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <t>&lt;button  v-bind:class="</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>{'btn-danger': !colorEdit || !baseSettings.editUserCurrentSetting}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "&gt; &lt;/button&gt;</t>
-    </r>
-  </si>
-  <si>
     <t>Подход 1</t>
   </si>
   <si>
@@ -2371,41 +2273,7 @@
     <t>несколько стилей</t>
   </si>
   <si>
-    <t>несколько стилей с условиями</t>
-  </si>
-  <si>
     <t>несколько стилей, комбинированных в объект</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">&lt;el-button </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:style="{
-  backgroundColor: item.length === 0 ? "#409EFF" : "#FFF", 
-  …
-}"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&gt; &lt;/el-button&gt;</t>
-    </r>
   </si>
   <si>
     <r>
@@ -2436,69 +2304,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  &gt; &lt;/el-button&gt;</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">&lt;button  v-bind:class=" </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>colorEdit  ? 'btn-danger' : null</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "&gt; &lt;/button&gt;</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">&lt;button 
-         v-bind:class="
-        [
-          </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">colorEdit ? 'btn-danger' : null ,
-          colorEdit ? 'btn-danger' : null </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-         ]
-       "
-&lt;/button&gt;</t>
     </r>
   </si>
   <si>
@@ -5945,17 +5750,455 @@
     }),</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">&lt;button  v-bind:class=" </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>colorEdit</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  ? 'btn-danger' : null</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "&gt; &lt;/button&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">&lt;button 
+         v-bind:class="
+        [
+          </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>colorEdit</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ? 'btn-danger' : null ,
+          </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>colorEdit</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ? 'btn-danger' : null </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+         ]
+       "
+&lt;/button&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">&lt;button 
+         v-bind:class="
+        {
+          </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">'btn-danger': </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>colorEdit &amp;&amp; baseSettings.editUserCurrentSetting</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">,
+          'btn-default': </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>!colorEdit || !baseSettings.editUserCurrentSetting</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, 
+          'btn-primary': </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>colorEdit &amp;&amp; !baseSettings.editUserCurrentSetting</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+         }
+       "
+&lt;/button&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">&lt;button 
+        v-bind:class="[
+           </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">'custom_class_1',
+            {'btn-danger': </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>!colorEdit || !baseSettings.editUserCurrentSetting</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">}, 
+           </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>colorEdit &amp;&amp; baseSettings.editUserCurrentSetting</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ? 'btn-danger' : null </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+         ]"
+&lt;/button&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">&lt;el-button </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:style="{
+  backgroundColor:</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> item.length === 0</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ? "#409EFF" : "#FFF", 
+  …
+}"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&gt; &lt;/el-button&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>один class</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (самый предпочтительный)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>&lt;button  v-bind:class="</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">{'btn-danger': </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>!colorEdit, ...</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "&gt; &lt;/button&gt;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">несколько стилей с условиями </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(самый предпочтительный)</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="30" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -6274,10 +6517,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -6288,20 +6531,20 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -6310,75 +6553,72 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="25" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="8" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="2" applyFill="1"/>
-    <xf numFmtId="49" fontId="9" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="49" fontId="10" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="9" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="10" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="10" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="11" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="11" borderId="0" xfId="2" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -6387,19 +6627,25 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -6408,7 +6654,7 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -6872,7 +7118,7 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -6888,51 +7134,51 @@
         <v>55</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A11" s="15" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="15" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A12" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="B12" s="47" t="s">
-        <v>287</v>
+        <v>151</v>
+      </c>
+      <c r="B12" s="45" t="s">
+        <v>280</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A13" s="15"/>
-      <c r="B13" s="47" t="s">
-        <v>288</v>
-      </c>
-      <c r="C13" s="47" t="s">
-        <v>289</v>
+      <c r="B13" s="45" t="s">
+        <v>281</v>
+      </c>
+      <c r="C13" s="45" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" s="15"/>
       <c r="B14" s="33" t="s">
-        <v>285</v>
-      </c>
-      <c r="C14" s="45" t="s">
-        <v>286</v>
+        <v>278</v>
+      </c>
+      <c r="C14" s="44" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.3">
@@ -6988,7 +7234,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="30" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B20" s="12"/>
       <c r="C20" s="9"/>
@@ -6998,10 +7244,10 @@
         <v>101</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>66</v>
@@ -7009,7 +7255,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="31" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
@@ -7018,10 +7264,10 @@
       <c r="A23" s="2"/>
       <c r="B23" s="15"/>
       <c r="C23" s="29" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -7247,13 +7493,13 @@
         <v>126</v>
       </c>
       <c r="B46" s="32" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="C46" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="D46" s="42" t="s">
-        <v>254</v>
+      <c r="D46" s="41" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="216" x14ac:dyDescent="0.3">
@@ -7266,8 +7512,8 @@
       <c r="C47" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="D47" s="42" t="s">
-        <v>280</v>
+      <c r="D47" s="41" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
@@ -7283,10 +7529,10 @@
         <v>20</v>
       </c>
       <c r="B49" s="15" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>19</v>
@@ -7297,10 +7543,10 @@
         <v>17</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>21</v>
@@ -7311,10 +7557,10 @@
         <v>16</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>22</v>
@@ -7325,10 +7571,10 @@
         <v>9</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>23</v>
@@ -7339,10 +7585,10 @@
         <v>18</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>24</v>
@@ -7353,10 +7599,10 @@
         <v>14</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>28</v>
@@ -7367,10 +7613,10 @@
         <v>131</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="D55" s="15"/>
     </row>
@@ -7379,13 +7625,13 @@
         <v>90</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="C56" s="15" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
@@ -7393,13 +7639,13 @@
         <v>133</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="C57" s="15" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -7407,10 +7653,10 @@
         <v>11</v>
       </c>
       <c r="B58" s="15" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="C58" s="15" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="D58" s="1" t="s">
         <v>25</v>
@@ -7421,10 +7667,10 @@
         <v>12</v>
       </c>
       <c r="B59" s="15" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C59" s="15" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>27</v>
@@ -7435,10 +7681,10 @@
         <v>10</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="D60" s="1" t="s">
         <v>26</v>
@@ -7449,16 +7695,16 @@
         <v>13</v>
       </c>
       <c r="B61" s="15" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="C61" s="15" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="D61" s="15"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="10" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="B62" s="15"/>
       <c r="C62" s="15"/>
@@ -7466,7 +7712,7 @@
     </row>
     <row r="63" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="C63" s="15" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D63" s="15"/>
     </row>
@@ -7475,10 +7721,10 @@
         <v>131</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="C64" s="29" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D64" s="15"/>
     </row>
@@ -7487,26 +7733,26 @@
         <v>90</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="D65" s="15"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="10" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="B66" s="15"/>
       <c r="C66" s="15"/>
       <c r="D66" s="15" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="30" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="9"/>
@@ -7516,10 +7762,10 @@
         <v>101</v>
       </c>
       <c r="B68" s="15" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="C68" s="15" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="D68" s="1" t="s">
         <v>66</v>
@@ -7527,7 +7773,7 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="31" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="B69" s="15"/>
       <c r="C69" s="15"/>
@@ -7536,15 +7782,15 @@
       <c r="A70" s="2"/>
       <c r="B70" s="15"/>
       <c r="C70" s="29" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="10" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B71" s="15"/>
       <c r="C71" s="15"/>
@@ -7554,229 +7800,229 @@
     </row>
     <row r="72" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C72" s="29" t="s">
         <v>206</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C72" s="29" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="73" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="C73" s="29" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="D73" s="2"/>
     </row>
     <row r="74" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="B74" s="29" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="C74" s="29" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="C75" s="29" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
     </row>
     <row r="76" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="C76" s="29" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="C77" s="29" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="C78" s="32" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="B79" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C79" s="29" t="s">
         <v>212</v>
-      </c>
-      <c r="C79" s="29" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="10" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="2"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="C82" s="9"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="C83" s="9"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="C84" s="9"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C85" s="9"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C86" s="9"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="C87" s="9"/>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
     </row>
     <row r="90" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A90" s="32" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="B90" s="32"/>
       <c r="C90" s="32" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="91" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A91" s="32" t="s">
+        <v>241</v>
+      </c>
+      <c r="B91" s="32" t="s">
         <v>248</v>
       </c>
-      <c r="B91" s="32" t="s">
-        <v>255</v>
-      </c>
       <c r="C91" s="32" t="s">
+        <v>242</v>
+      </c>
+      <c r="D91" s="32" t="s">
         <v>249</v>
-      </c>
-      <c r="D91" s="32" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="B92" s="32" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="B95" s="32" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C95" s="32" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="C96" s="33" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="34" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="D97" s="1" t="s">
         <v>30</v>
@@ -7787,10 +8033,10 @@
         <v>131</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="C98" s="32" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
@@ -7798,24 +8044,24 @@
         <v>90</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="10" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
     </row>
     <row r="103" spans="1:4" ht="144" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="C103" s="44" t="s">
-        <v>282</v>
+        <v>277</v>
+      </c>
+      <c r="C103" s="43" t="s">
+        <v>275</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="17" type="noConversion"/>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -7860,10 +8106,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A1" s="46"/>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
+      <c r="A1" s="47"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="22"/>
@@ -7894,7 +8140,7 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="P4" s="19"/>
       <c r="U4" s="19"/>
@@ -7903,27 +8149,27 @@
     <row r="5" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>149</v>
+        <v>290</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>287</v>
       </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>134</v>
@@ -7934,7 +8180,7 @@
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="15"/>
@@ -7942,61 +8188,61 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>151</v>
+        <v>136</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>283</v>
       </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>142</v>
+        <v>288</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>289</v>
       </c>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:22" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C11" s="35" t="s">
-        <v>152</v>
+        <v>146</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>284</v>
       </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>135</v>
+        <v>147</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>285</v>
       </c>
       <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>136</v>
+        <v>137</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>286</v>
       </c>
       <c r="D13" s="1"/>
     </row>
@@ -8005,10 +8251,10 @@
         <v>118</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C14" s="20" t="s">
         <v>139</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -8093,13 +8339,13 @@
     </row>
     <row r="6" spans="1:22" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B6" s="32" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
@@ -8109,13 +8355,13 @@
     </row>
     <row r="8" spans="1:22" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B8" s="32" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
@@ -8125,38 +8371,38 @@
     </row>
     <row r="10" spans="1:22" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="C10" s="36" t="s">
-        <v>270</v>
+        <v>264</v>
+      </c>
+      <c r="C10" s="35" t="s">
+        <v>263</v>
       </c>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:22" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="C11" s="36" t="s">
-        <v>273</v>
+        <v>268</v>
+      </c>
+      <c r="C11" s="35" t="s">
+        <v>266</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="144" x14ac:dyDescent="0.3">
       <c r="B12" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="C12" s="36" t="s">
-        <v>274</v>
+        <v>269</v>
+      </c>
+      <c r="C12" s="35" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="288" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="C13" s="36" t="s">
-        <v>278</v>
+        <v>270</v>
+      </c>
+      <c r="C13" s="35" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
@@ -8227,7 +8473,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C30:D44">
     <sortCondition ref="D30:D44"/>
   </sortState>
-  <phoneticPr fontId="17" type="noConversion"/>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
@@ -8282,96 +8528,96 @@
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>279</v>
-      </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="37"/>
+        <v>272</v>
+      </c>
+      <c r="B3" s="37"/>
+      <c r="C3" s="36"/>
       <c r="P3" s="1"/>
       <c r="U3" s="1"/>
       <c r="V3" s="2"/>
     </row>
     <row r="4" spans="1:22" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="38"/>
-      <c r="B4" s="38"/>
-      <c r="C4" s="43" t="s">
-        <v>281</v>
+      <c r="A4" s="37"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="42" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A5" s="37"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="39"/>
+      <c r="A5" s="36"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="38"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A6" s="37"/>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
+      <c r="A6" s="36"/>
+      <c r="B6" s="39"/>
+      <c r="C6" s="39"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A7" s="37"/>
-      <c r="B7" s="38"/>
-      <c r="C7" s="39"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="38"/>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A8" s="37"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
+      <c r="A8" s="36"/>
+      <c r="B8" s="39"/>
+      <c r="C8" s="39"/>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A9" s="37"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="39"/>
+      <c r="A9" s="36"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="38"/>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A10" s="37"/>
-      <c r="B10" s="38"/>
-      <c r="C10" s="41"/>
+      <c r="A10" s="36"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="40"/>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A11" s="37"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="41"/>
+      <c r="A11" s="36"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="40"/>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A12" s="37"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="41"/>
+      <c r="A12" s="36"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="40"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A13" s="37"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="41"/>
+      <c r="A13" s="36"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="40"/>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A14" s="37"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="39"/>
+      <c r="A14" s="36"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="38"/>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A15" s="37"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="39"/>
+      <c r="A15" s="36"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="38"/>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A16" s="37"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="39"/>
+      <c r="A16" s="36"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="38"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="37"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="39"/>
+      <c r="A17" s="36"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="38"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="37"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="39"/>
+      <c r="A18" s="36"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="38"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="37"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="39"/>
+      <c r="A19" s="36"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="38"/>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
       <c r="C38" s="27" t="s">

</xml_diff>